<commit_message>
adding VENV_DIR to .gitignore etc
</commit_message>
<xml_diff>
--- a/data/exchange_rates/USD_CZK.xlsx
+++ b/data/exchange_rates/USD_CZK.xlsx
@@ -429,26 +429,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>CZK= (BID)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Returns</t>
         </is>
@@ -456,511 +451,449 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>44928</v>
-      </c>
-      <c r="D2" t="n">
-        <v>22.352</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-0.008956282699299378</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>34337</v>
+      </c>
+      <c r="C2" t="n">
+        <v>27.93</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>44564</v>
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>34701</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26.661</v>
       </c>
       <c r="D3" t="n">
-        <v>22.554</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.03226692297130296</v>
+        <v>-0.0454</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>44197</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>35066</v>
+      </c>
+      <c r="C4" t="n">
+        <v>27.213</v>
       </c>
       <c r="D4" t="n">
-        <v>21.849</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.01874388026297389</v>
+        <v>0.0207</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>43831</v>
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>35432</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34.657</v>
       </c>
       <c r="D5" t="n">
-        <v>21.447</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-0.05361397934868943</v>
+        <v>0.2735</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>43466</v>
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>35797</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29.957</v>
       </c>
       <c r="D6" t="n">
-        <v>22.662</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.01101940664733437</v>
+        <v>-0.1356</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>43101</v>
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>36164</v>
+      </c>
+      <c r="C7" t="n">
+        <v>35.79</v>
       </c>
       <c r="D7" t="n">
-        <v>22.415</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.05343547325876494</v>
+        <v>0.1947</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>9</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>42737</v>
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>36528</v>
+      </c>
+      <c r="C8" t="n">
+        <v>37.602</v>
       </c>
       <c r="D8" t="n">
-        <v>21.278</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-0.1703836556456644</v>
+        <v>0.0506</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>42370</v>
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>36893</v>
+      </c>
+      <c r="C9" t="n">
+        <v>35.578</v>
       </c>
       <c r="D9" t="n">
-        <v>25.648</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.03165600740115036</v>
+        <v>-0.0538</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="n">
-        <v>11</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>42005</v>
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>37258</v>
+      </c>
+      <c r="C10" t="n">
+        <v>30.041</v>
       </c>
       <c r="D10" t="n">
-        <v>24.861</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.08886650315346881</v>
+        <v>-0.1556</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="n">
-        <v>12</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>41640</v>
+        <v>9</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>37622</v>
+      </c>
+      <c r="C11" t="n">
+        <v>25.672</v>
       </c>
       <c r="D11" t="n">
-        <v>22.832</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.1493003120910098</v>
+        <v>-0.1454</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="n">
-        <v>13</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>41275</v>
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>37987</v>
+      </c>
+      <c r="C12" t="n">
+        <v>22.415</v>
       </c>
       <c r="D12" t="n">
-        <v>19.866</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.04640505662365026</v>
+        <v>-0.1269</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="n">
-        <v>14</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>40910</v>
+        <v>11</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>38355</v>
+      </c>
+      <c r="C13" t="n">
+        <v>24.534</v>
       </c>
       <c r="D13" t="n">
-        <v>18.985</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-0.03785728765457125</v>
+        <v>0.0945</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>40546</v>
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>38719</v>
+      </c>
+      <c r="C14" t="n">
+        <v>20.82</v>
       </c>
       <c r="D14" t="n">
-        <v>19.732</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.05699592886222413</v>
+        <v>-0.1514</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="n">
-        <v>16</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>40179</v>
+        <v>13</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>39083</v>
+      </c>
+      <c r="C15" t="n">
+        <v>18.168</v>
       </c>
       <c r="D15" t="n">
-        <v>18.668</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.01583501115524843</v>
+        <v>-0.1274</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="n">
-        <v>17</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>39814</v>
+        <v>14</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>39448</v>
+      </c>
+      <c r="C16" t="n">
+        <v>19.114</v>
       </c>
       <c r="D16" t="n">
-        <v>18.377</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-0.03855812493460301</v>
+        <v>0.0521</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="n">
-        <v>18</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>39448</v>
+        <v>15</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>39814</v>
+      </c>
+      <c r="C17" t="n">
+        <v>18.377</v>
       </c>
       <c r="D17" t="n">
-        <v>19.114</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.05206957287538538</v>
+        <v>-0.0386</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="n">
-        <v>19</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>39083</v>
+        <v>16</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>40179</v>
+      </c>
+      <c r="C18" t="n">
+        <v>18.668</v>
       </c>
       <c r="D18" t="n">
-        <v>18.168</v>
-      </c>
-      <c r="E18" t="n">
-        <v>-0.1273775216138329</v>
+        <v>0.0158</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="n">
-        <v>20</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>38719</v>
+        <v>17</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>40546</v>
+      </c>
+      <c r="C19" t="n">
+        <v>19.732</v>
       </c>
       <c r="D19" t="n">
-        <v>20.82</v>
-      </c>
-      <c r="E19" t="n">
-        <v>-0.1513817559305453</v>
+        <v>0.057</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="n">
-        <v>21</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>38355</v>
+        <v>18</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>40910</v>
+      </c>
+      <c r="C20" t="n">
+        <v>18.985</v>
       </c>
       <c r="D20" t="n">
-        <v>24.534</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.09453490965871068</v>
+        <v>-0.0379</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="n">
-        <v>22</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>37987</v>
+        <v>19</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>41275</v>
+      </c>
+      <c r="C21" t="n">
+        <v>19.866</v>
       </c>
       <c r="D21" t="n">
-        <v>22.415</v>
-      </c>
-      <c r="E21" t="n">
-        <v>-0.1268697413524463</v>
+        <v>0.0464</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="n">
-        <v>23</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>37622</v>
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>41640</v>
+      </c>
+      <c r="C22" t="n">
+        <v>22.832</v>
       </c>
       <c r="D22" t="n">
-        <v>25.672</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-0.1454345727505742</v>
+        <v>0.1493</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="n">
-        <v>24</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>37258</v>
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>42005</v>
+      </c>
+      <c r="C23" t="n">
+        <v>24.861</v>
       </c>
       <c r="D23" t="n">
-        <v>30.041</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-0.1556298836359549</v>
+        <v>0.08890000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="n">
-        <v>25</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>36893</v>
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>42370</v>
+      </c>
+      <c r="C24" t="n">
+        <v>25.648</v>
       </c>
       <c r="D24" t="n">
-        <v>35.578</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-0.05382692409978176</v>
+        <v>0.0317</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="n">
-        <v>26</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>36528</v>
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>42737</v>
+      </c>
+      <c r="C25" t="n">
+        <v>21.278</v>
       </c>
       <c r="D25" t="n">
-        <v>37.602</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.05062866722548191</v>
+        <v>-0.1704</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="n">
-        <v>27</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>36164</v>
+        <v>24</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>43101</v>
+      </c>
+      <c r="C26" t="n">
+        <v>22.415</v>
       </c>
       <c r="D26" t="n">
-        <v>35.79</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.1947124211369629</v>
+        <v>0.0534</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="n">
-        <v>28</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>35797</v>
+        <v>25</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>43466</v>
+      </c>
+      <c r="C27" t="n">
+        <v>22.662</v>
       </c>
       <c r="D27" t="n">
-        <v>29.957</v>
-      </c>
-      <c r="E27" t="n">
-        <v>-0.1356147387252213</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="n">
-        <v>29</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>35432</v>
+        <v>26</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>43831</v>
+      </c>
+      <c r="C28" t="n">
+        <v>21.447</v>
       </c>
       <c r="D28" t="n">
-        <v>34.657</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0.2735457318193509</v>
+        <v>-0.0536</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="n">
-        <v>30</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>35066</v>
+        <v>27</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>44197</v>
+      </c>
+      <c r="C29" t="n">
+        <v>21.849</v>
       </c>
       <c r="D29" t="n">
-        <v>27.213</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0.02070439968493303</v>
+        <v>0.0187</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="n">
-        <v>31</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>34701</v>
+        <v>28</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>44564</v>
+      </c>
+      <c r="C30" t="n">
+        <v>22.554</v>
       </c>
       <c r="D30" t="n">
-        <v>26.661</v>
-      </c>
-      <c r="E30" t="n">
-        <v>-0.04543501611170778</v>
+        <v>0.0323</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>44928</v>
+      </c>
+      <c r="C31" t="n">
+        <v>22.352</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="n">
-        <v>32</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>34337</v>
-      </c>
-      <c r="D31" t="n">
-        <v>27.93</v>
-      </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="B32" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="C32" t="n">
+        <v>24.324</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.0882</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>45658</v>
+      </c>
+      <c r="C33" t="n">
+        <v>23.975</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.0143</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>